<commit_message>
debug adb save model
</commit_message>
<xml_diff>
--- a/results/openset_pivot.xlsx
+++ b/results/openset_pivot.xlsx
@@ -2138,10 +2138,18 @@
       <c r="W16" t="n">
         <v>0.9096437880104256</v>
       </c>
-      <c r="X16" t="inlineStr"/>
-      <c r="Y16" t="inlineStr"/>
-      <c r="Z16" t="inlineStr"/>
-      <c r="AA16" t="inlineStr"/>
+      <c r="X16" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>0.8937408390564399</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>0.8999289725841433</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>0.8009188361408882</v>
+      </c>
       <c r="AB16" t="n">
         <v>0.9675</v>
       </c>
@@ -2166,10 +2174,18 @@
       <c r="AI16" t="n">
         <v>0.9570383912248628</v>
       </c>
-      <c r="AJ16" t="inlineStr"/>
-      <c r="AK16" t="inlineStr"/>
-      <c r="AL16" t="inlineStr"/>
-      <c r="AM16" t="inlineStr"/>
+      <c r="AJ16" t="n">
+        <v>0.9685</v>
+      </c>
+      <c r="AK16" t="n">
+        <v>0.976709440243004</v>
+      </c>
+      <c r="AL16" t="n">
+        <v>0.9789439319309808</v>
+      </c>
+      <c r="AM16" t="n">
+        <v>0.9431920649233544</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n"/>
@@ -2237,10 +2253,18 @@
       <c r="W17" t="n">
         <v>0.8901239846088072</v>
       </c>
-      <c r="X17" t="inlineStr"/>
-      <c r="Y17" t="inlineStr"/>
-      <c r="Z17" t="inlineStr"/>
-      <c r="AA17" t="inlineStr"/>
+      <c r="X17" t="n">
+        <v>0.895</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>0.9154337885245184</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>0.9210139898107688</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>0.8317307692307693</v>
+      </c>
       <c r="AB17" t="n">
         <v>0.9885</v>
       </c>
@@ -2265,10 +2289,18 @@
       <c r="AI17" t="n">
         <v>0.9793038570084666</v>
       </c>
-      <c r="AJ17" t="inlineStr"/>
-      <c r="AK17" t="inlineStr"/>
-      <c r="AL17" t="inlineStr"/>
-      <c r="AM17" t="inlineStr"/>
+      <c r="AJ17" t="n">
+        <v>0.9535</v>
+      </c>
+      <c r="AK17" t="n">
+        <v>0.9635020514235886</v>
+      </c>
+      <c r="AL17" t="n">
+        <v>0.9665507292992196</v>
+      </c>
+      <c r="AM17" t="n">
+        <v>0.9177718832891246</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n"/>
@@ -2324,14 +2356,30 @@
       <c r="S18" t="n">
         <v>0.9431711145996859</v>
       </c>
-      <c r="T18" t="inlineStr"/>
-      <c r="U18" t="inlineStr"/>
-      <c r="V18" t="inlineStr"/>
-      <c r="W18" t="inlineStr"/>
-      <c r="X18" t="inlineStr"/>
-      <c r="Y18" t="inlineStr"/>
-      <c r="Z18" t="inlineStr"/>
-      <c r="AA18" t="inlineStr"/>
+      <c r="T18" t="n">
+        <v>0.8925</v>
+      </c>
+      <c r="U18" t="n">
+        <v>0.8833001430703827</v>
+      </c>
+      <c r="V18" t="n">
+        <v>0.8815152148486854</v>
+      </c>
+      <c r="W18" t="n">
+        <v>0.9011494252873564</v>
+      </c>
+      <c r="X18" t="n">
+        <v>0.9175</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>0.9369200077183196</v>
+      </c>
+      <c r="Z18" t="n">
+        <v>0.9429282310741</v>
+      </c>
+      <c r="AA18" t="n">
+        <v>0.8467966573816156</v>
+      </c>
       <c r="AB18" t="n">
         <v>0.992</v>
       </c>
@@ -2344,14 +2392,30 @@
       <c r="AE18" t="n">
         <v>0.9947019867549668</v>
       </c>
-      <c r="AF18" t="inlineStr"/>
-      <c r="AG18" t="inlineStr"/>
-      <c r="AH18" t="inlineStr"/>
-      <c r="AI18" t="inlineStr"/>
-      <c r="AJ18" t="inlineStr"/>
-      <c r="AK18" t="inlineStr"/>
-      <c r="AL18" t="inlineStr"/>
-      <c r="AM18" t="inlineStr"/>
+      <c r="AF18" t="n">
+        <v>0.9605</v>
+      </c>
+      <c r="AG18" t="n">
+        <v>0.9591789085531396</v>
+      </c>
+      <c r="AH18" t="n">
+        <v>0.9589712476674036</v>
+      </c>
+      <c r="AI18" t="n">
+        <v>0.9612555174104952</v>
+      </c>
+      <c r="AJ18" t="n">
+        <v>0.9595</v>
+      </c>
+      <c r="AK18" t="n">
+        <v>0.9692629935669244</v>
+      </c>
+      <c r="AL18" t="n">
+        <v>0.9726519262699764</v>
+      </c>
+      <c r="AM18" t="n">
+        <v>0.918429003021148</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n"/>
@@ -2395,30 +2459,78 @@
       <c r="O19" t="n">
         <v>0.5337078651685393</v>
       </c>
-      <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="inlineStr"/>
-      <c r="S19" t="inlineStr"/>
-      <c r="T19" t="inlineStr"/>
-      <c r="U19" t="inlineStr"/>
-      <c r="V19" t="inlineStr"/>
-      <c r="W19" t="inlineStr"/>
-      <c r="X19" t="inlineStr"/>
-      <c r="Y19" t="inlineStr"/>
-      <c r="Z19" t="inlineStr"/>
-      <c r="AA19" t="inlineStr"/>
-      <c r="AB19" t="inlineStr"/>
-      <c r="AC19" t="inlineStr"/>
-      <c r="AD19" t="inlineStr"/>
-      <c r="AE19" t="inlineStr"/>
-      <c r="AF19" t="inlineStr"/>
-      <c r="AG19" t="inlineStr"/>
-      <c r="AH19" t="inlineStr"/>
-      <c r="AI19" t="inlineStr"/>
-      <c r="AJ19" t="inlineStr"/>
-      <c r="AK19" t="inlineStr"/>
-      <c r="AL19" t="inlineStr"/>
-      <c r="AM19" t="inlineStr"/>
+      <c r="P19" t="n">
+        <v>0.954</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>0.9135475922098584</v>
+      </c>
+      <c r="R19" t="n">
+        <v>0.902289897537076</v>
+      </c>
+      <c r="S19" t="n">
+        <v>0.9698360655737704</v>
+      </c>
+      <c r="T19" t="n">
+        <v>0.9005</v>
+      </c>
+      <c r="U19" t="n">
+        <v>0.8927419605149616</v>
+      </c>
+      <c r="V19" t="n">
+        <v>0.8914608646822619</v>
+      </c>
+      <c r="W19" t="n">
+        <v>0.9055529188419554</v>
+      </c>
+      <c r="X19" t="n">
+        <v>0.8575</v>
+      </c>
+      <c r="Y19" t="n">
+        <v>0.8842973300320611</v>
+      </c>
+      <c r="Z19" t="n">
+        <v>0.8919684340854805</v>
+      </c>
+      <c r="AA19" t="n">
+        <v>0.7692307692307693</v>
+      </c>
+      <c r="AB19" t="n">
+        <v>0.9575</v>
+      </c>
+      <c r="AC19" t="n">
+        <v>0.9186120529762056</v>
+      </c>
+      <c r="AD19" t="n">
+        <v>0.907921055750218</v>
+      </c>
+      <c r="AE19" t="n">
+        <v>0.9720670391061452</v>
+      </c>
+      <c r="AF19" t="n">
+        <v>0.9465</v>
+      </c>
+      <c r="AG19" t="n">
+        <v>0.945134354103176</v>
+      </c>
+      <c r="AH19" t="n">
+        <v>0.9449579632107644</v>
+      </c>
+      <c r="AI19" t="n">
+        <v>0.9468982630272952</v>
+      </c>
+      <c r="AJ19" t="n">
+        <v>0.947</v>
+      </c>
+      <c r="AK19" t="n">
+        <v>0.959201996691999</v>
+      </c>
+      <c r="AL19" t="n">
+        <v>0.9631740489967182</v>
+      </c>
+      <c r="AM19" t="n">
+        <v>0.8996212121212122</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n"/>
@@ -6368,10 +6480,18 @@
       <c r="C54" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="D54" t="inlineStr"/>
-      <c r="E54" t="inlineStr"/>
-      <c r="F54" t="inlineStr"/>
-      <c r="G54" t="inlineStr"/>
+      <c r="D54" t="n">
+        <v>67.34999999999999</v>
+      </c>
+      <c r="E54" t="n">
+        <v>14.5098</v>
+      </c>
+      <c r="F54" t="n">
+        <v>13.3144</v>
+      </c>
+      <c r="G54" t="n">
+        <v>80.2568</v>
+      </c>
       <c r="H54" t="n">
         <v>66.40000000000001</v>
       </c>
@@ -11230,10 +11350,18 @@
       <c r="C96" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D96" t="inlineStr"/>
-      <c r="E96" t="inlineStr"/>
-      <c r="F96" t="inlineStr"/>
-      <c r="G96" t="inlineStr"/>
+      <c r="D96" t="n">
+        <v>13.88</v>
+      </c>
+      <c r="E96" t="n">
+        <v>12.5681</v>
+      </c>
+      <c r="F96" t="n">
+        <v>12.6525</v>
+      </c>
+      <c r="G96" t="n">
+        <v>11.5556</v>
+      </c>
       <c r="H96" t="n">
         <v>20.61</v>
       </c>
@@ -11337,14 +11465,30 @@
       <c r="C97" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D97" t="inlineStr"/>
-      <c r="E97" t="inlineStr"/>
-      <c r="F97" t="inlineStr"/>
-      <c r="G97" t="inlineStr"/>
-      <c r="H97" t="inlineStr"/>
-      <c r="I97" t="inlineStr"/>
-      <c r="J97" t="inlineStr"/>
-      <c r="K97" t="inlineStr"/>
+      <c r="D97" t="n">
+        <v>12.86</v>
+      </c>
+      <c r="E97" t="n">
+        <v>14.8782</v>
+      </c>
+      <c r="F97" t="n">
+        <v>14.7854</v>
+      </c>
+      <c r="G97" t="n">
+        <v>15.8996</v>
+      </c>
+      <c r="H97" t="n">
+        <v>17.55</v>
+      </c>
+      <c r="I97" t="n">
+        <v>15.0822</v>
+      </c>
+      <c r="J97" t="n">
+        <v>14.8466</v>
+      </c>
+      <c r="K97" t="n">
+        <v>20.5011</v>
+      </c>
       <c r="L97" t="n">
         <v>56.53</v>
       </c>
@@ -11436,10 +11580,18 @@
       <c r="C98" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="D98" t="inlineStr"/>
-      <c r="E98" t="inlineStr"/>
-      <c r="F98" t="inlineStr"/>
-      <c r="G98" t="inlineStr"/>
+      <c r="D98" t="n">
+        <v>40</v>
+      </c>
+      <c r="E98" t="n">
+        <v>13.6643</v>
+      </c>
+      <c r="F98" t="n">
+        <v>9.789300000000001</v>
+      </c>
+      <c r="G98" t="n">
+        <v>56.2893</v>
+      </c>
       <c r="H98" t="n">
         <v>32.04</v>
       </c>
@@ -31935,10 +32087,18 @@
       <c r="C275" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="D275" t="inlineStr"/>
-      <c r="E275" t="inlineStr"/>
-      <c r="F275" t="inlineStr"/>
-      <c r="G275" t="inlineStr"/>
+      <c r="D275" t="n">
+        <v>67.09999999999999</v>
+      </c>
+      <c r="E275" t="n">
+        <v>65.3908</v>
+      </c>
+      <c r="F275" t="n">
+        <v>65.27809999999999</v>
+      </c>
+      <c r="G275" t="n">
+        <v>66.2921</v>
+      </c>
       <c r="H275" t="n">
         <v>67.75</v>
       </c>
@@ -32042,18 +32202,42 @@
       <c r="C276" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D276" t="inlineStr"/>
-      <c r="E276" t="inlineStr"/>
-      <c r="F276" t="inlineStr"/>
-      <c r="G276" t="inlineStr"/>
-      <c r="H276" t="inlineStr"/>
-      <c r="I276" t="inlineStr"/>
-      <c r="J276" t="inlineStr"/>
-      <c r="K276" t="inlineStr"/>
-      <c r="L276" t="inlineStr"/>
-      <c r="M276" t="inlineStr"/>
-      <c r="N276" t="inlineStr"/>
-      <c r="O276" t="inlineStr"/>
+      <c r="D276" t="n">
+        <v>41.87</v>
+      </c>
+      <c r="E276" t="n">
+        <v>26.257</v>
+      </c>
+      <c r="F276" t="n">
+        <v>23.0223</v>
+      </c>
+      <c r="G276" t="n">
+        <v>52.1348</v>
+      </c>
+      <c r="H276" t="n">
+        <v>33.55</v>
+      </c>
+      <c r="I276" t="n">
+        <v>43.2631</v>
+      </c>
+      <c r="J276" t="n">
+        <v>44.6205</v>
+      </c>
+      <c r="K276" t="n">
+        <v>21.544</v>
+      </c>
+      <c r="L276" t="n">
+        <v>41.87</v>
+      </c>
+      <c r="M276" t="n">
+        <v>44.4045</v>
+      </c>
+      <c r="N276" t="n">
+        <v>44.9889</v>
+      </c>
+      <c r="O276" t="n">
+        <v>30.9623</v>
+      </c>
       <c r="P276" t="n">
         <v>87.26000000000001</v>
       </c>
@@ -32133,18 +32317,42 @@
       <c r="C277" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D277" t="inlineStr"/>
-      <c r="E277" t="inlineStr"/>
-      <c r="F277" t="inlineStr"/>
-      <c r="G277" t="inlineStr"/>
-      <c r="H277" t="inlineStr"/>
-      <c r="I277" t="inlineStr"/>
-      <c r="J277" t="inlineStr"/>
-      <c r="K277" t="inlineStr"/>
-      <c r="L277" t="inlineStr"/>
-      <c r="M277" t="inlineStr"/>
-      <c r="N277" t="inlineStr"/>
-      <c r="O277" t="inlineStr"/>
+      <c r="D277" t="n">
+        <v>84.66</v>
+      </c>
+      <c r="E277" t="n">
+        <v>37.408</v>
+      </c>
+      <c r="F277" t="n">
+        <v>30.5326</v>
+      </c>
+      <c r="G277" t="n">
+        <v>92.4117</v>
+      </c>
+      <c r="H277" t="n">
+        <v>43.43</v>
+      </c>
+      <c r="I277" t="n">
+        <v>39.9571</v>
+      </c>
+      <c r="J277" t="n">
+        <v>39.6664</v>
+      </c>
+      <c r="K277" t="n">
+        <v>44.6086</v>
+      </c>
+      <c r="L277" t="n">
+        <v>47.33</v>
+      </c>
+      <c r="M277" t="n">
+        <v>43.1468</v>
+      </c>
+      <c r="N277" t="n">
+        <v>43.6684</v>
+      </c>
+      <c r="O277" t="n">
+        <v>31.1512</v>
+      </c>
       <c r="P277" t="n">
         <v>45.38</v>
       </c>
@@ -32224,14 +32432,30 @@
       <c r="C278" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="D278" t="inlineStr"/>
-      <c r="E278" t="inlineStr"/>
-      <c r="F278" t="inlineStr"/>
-      <c r="G278" t="inlineStr"/>
-      <c r="H278" t="inlineStr"/>
-      <c r="I278" t="inlineStr"/>
-      <c r="J278" t="inlineStr"/>
-      <c r="K278" t="inlineStr"/>
+      <c r="D278" t="n">
+        <v>44.86</v>
+      </c>
+      <c r="E278" t="n">
+        <v>40.2369</v>
+      </c>
+      <c r="F278" t="n">
+        <v>38.8733</v>
+      </c>
+      <c r="G278" t="n">
+        <v>51.146</v>
+      </c>
+      <c r="H278" t="n">
+        <v>52.54</v>
+      </c>
+      <c r="I278" t="n">
+        <v>43.4439</v>
+      </c>
+      <c r="J278" t="n">
+        <v>43.0034</v>
+      </c>
+      <c r="K278" t="n">
+        <v>50.4918</v>
+      </c>
       <c r="L278" t="n">
         <v>63.2</v>
       </c>
@@ -32323,10 +32547,18 @@
       <c r="C279" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="D279" t="inlineStr"/>
-      <c r="E279" t="inlineStr"/>
-      <c r="F279" t="inlineStr"/>
-      <c r="G279" t="inlineStr"/>
+      <c r="D279" t="n">
+        <v>45.25</v>
+      </c>
+      <c r="E279" t="n">
+        <v>23.2932</v>
+      </c>
+      <c r="F279" t="n">
+        <v>18.7791</v>
+      </c>
+      <c r="G279" t="n">
+        <v>59.4059</v>
+      </c>
       <c r="H279" t="inlineStr"/>
       <c r="I279" t="inlineStr"/>
       <c r="J279" t="inlineStr"/>
@@ -32343,10 +32575,18 @@
       <c r="O279" t="n">
         <v>63.2143</v>
       </c>
-      <c r="P279" t="inlineStr"/>
-      <c r="Q279" t="inlineStr"/>
-      <c r="R279" t="inlineStr"/>
-      <c r="S279" t="inlineStr"/>
+      <c r="P279" t="n">
+        <v>51.37</v>
+      </c>
+      <c r="Q279" t="n">
+        <v>33.0077</v>
+      </c>
+      <c r="R279" t="n">
+        <v>29.0807</v>
+      </c>
+      <c r="S279" t="n">
+        <v>64.42310000000001</v>
+      </c>
       <c r="T279" t="n">
         <v>88.3</v>
       </c>
@@ -35773,10 +36013,18 @@
       <c r="C309" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="D309" t="inlineStr"/>
-      <c r="E309" t="inlineStr"/>
-      <c r="F309" t="inlineStr"/>
-      <c r="G309" t="inlineStr"/>
+      <c r="D309" t="n">
+        <v>0.035064935064935</v>
+      </c>
+      <c r="E309" t="n">
+        <v>0.0421853943949084</v>
+      </c>
+      <c r="F309" t="n">
+        <v>0.0470967741935483</v>
+      </c>
+      <c r="G309" t="n">
+        <v>0.0028943560057887</v>
+      </c>
       <c r="H309" t="n">
         <v>0.122077922077922</v>
       </c>
@@ -42261,18 +42509,42 @@
       <c r="C365" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="D365" t="inlineStr"/>
-      <c r="E365" t="inlineStr"/>
-      <c r="F365" t="inlineStr"/>
-      <c r="G365" t="inlineStr"/>
-      <c r="H365" t="inlineStr"/>
-      <c r="I365" t="inlineStr"/>
-      <c r="J365" t="inlineStr"/>
-      <c r="K365" t="inlineStr"/>
-      <c r="L365" t="inlineStr"/>
-      <c r="M365" t="inlineStr"/>
-      <c r="N365" t="inlineStr"/>
-      <c r="O365" t="inlineStr"/>
+      <c r="D365" t="n">
+        <v>32.63</v>
+      </c>
+      <c r="E365" t="n">
+        <v>38.555</v>
+      </c>
+      <c r="F365" t="n">
+        <v>40.0985</v>
+      </c>
+      <c r="G365" t="n">
+        <v>32.381</v>
+      </c>
+      <c r="H365" t="n">
+        <v>45.62</v>
+      </c>
+      <c r="I365" t="n">
+        <v>55.4078</v>
+      </c>
+      <c r="J365" t="n">
+        <v>57.5574</v>
+      </c>
+      <c r="K365" t="n">
+        <v>38.2114</v>
+      </c>
+      <c r="L365" t="n">
+        <v>42.3</v>
+      </c>
+      <c r="M365" t="n">
+        <v>49.773</v>
+      </c>
+      <c r="N365" t="n">
+        <v>53.6177</v>
+      </c>
+      <c r="O365" t="n">
+        <v>3.6364</v>
+      </c>
       <c r="P365" t="n">
         <v>62.84</v>
       </c>
@@ -42352,18 +42624,42 @@
       <c r="C366" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D366" t="inlineStr"/>
-      <c r="E366" t="inlineStr"/>
-      <c r="F366" t="inlineStr"/>
-      <c r="G366" t="inlineStr"/>
-      <c r="H366" t="inlineStr"/>
-      <c r="I366" t="inlineStr"/>
-      <c r="J366" t="inlineStr"/>
-      <c r="K366" t="inlineStr"/>
-      <c r="L366" t="inlineStr"/>
-      <c r="M366" t="inlineStr"/>
-      <c r="N366" t="inlineStr"/>
-      <c r="O366" t="inlineStr"/>
+      <c r="D366" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="E366" t="n">
+        <v>43.5106</v>
+      </c>
+      <c r="F366" t="n">
+        <v>42.1375</v>
+      </c>
+      <c r="G366" t="n">
+        <v>49.0028</v>
+      </c>
+      <c r="H366" t="n">
+        <v>45.92</v>
+      </c>
+      <c r="I366" t="n">
+        <v>22.2452</v>
+      </c>
+      <c r="J366" t="n">
+        <v>17.6409</v>
+      </c>
+      <c r="K366" t="n">
+        <v>59.0799</v>
+      </c>
+      <c r="L366" t="n">
+        <v>41.69</v>
+      </c>
+      <c r="M366" t="n">
+        <v>44.7288</v>
+      </c>
+      <c r="N366" t="n">
+        <v>45.9275</v>
+      </c>
+      <c r="O366" t="n">
+        <v>30.3448</v>
+      </c>
       <c r="P366" t="n">
         <v>36.86</v>
       </c>
@@ -42443,18 +42739,42 @@
       <c r="C367" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D367" t="inlineStr"/>
-      <c r="E367" t="inlineStr"/>
-      <c r="F367" t="inlineStr"/>
-      <c r="G367" t="inlineStr"/>
-      <c r="H367" t="inlineStr"/>
-      <c r="I367" t="inlineStr"/>
-      <c r="J367" t="inlineStr"/>
-      <c r="K367" t="inlineStr"/>
-      <c r="L367" t="inlineStr"/>
-      <c r="M367" t="inlineStr"/>
-      <c r="N367" t="inlineStr"/>
-      <c r="O367" t="inlineStr"/>
+      <c r="D367" t="n">
+        <v>47.13</v>
+      </c>
+      <c r="E367" t="n">
+        <v>44.6968</v>
+      </c>
+      <c r="F367" t="n">
+        <v>41.9083</v>
+      </c>
+      <c r="G367" t="n">
+        <v>55.8511</v>
+      </c>
+      <c r="H367" t="n">
+        <v>42.3</v>
+      </c>
+      <c r="I367" t="n">
+        <v>44.5855</v>
+      </c>
+      <c r="J367" t="n">
+        <v>44.6251</v>
+      </c>
+      <c r="K367" t="n">
+        <v>44.2688</v>
+      </c>
+      <c r="L367" t="n">
+        <v>44.41</v>
+      </c>
+      <c r="M367" t="n">
+        <v>49.8753</v>
+      </c>
+      <c r="N367" t="n">
+        <v>51.6506</v>
+      </c>
+      <c r="O367" t="n">
+        <v>28.5714</v>
+      </c>
       <c r="P367" t="n">
         <v>43.81</v>
       </c>
@@ -42534,18 +42854,42 @@
       <c r="C368" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="D368" t="inlineStr"/>
-      <c r="E368" t="inlineStr"/>
-      <c r="F368" t="inlineStr"/>
-      <c r="G368" t="inlineStr"/>
-      <c r="H368" t="inlineStr"/>
-      <c r="I368" t="inlineStr"/>
-      <c r="J368" t="inlineStr"/>
-      <c r="K368" t="inlineStr"/>
-      <c r="L368" t="inlineStr"/>
-      <c r="M368" t="inlineStr"/>
-      <c r="N368" t="inlineStr"/>
-      <c r="O368" t="inlineStr"/>
+      <c r="D368" t="n">
+        <v>39.27</v>
+      </c>
+      <c r="E368" t="n">
+        <v>34.8961</v>
+      </c>
+      <c r="F368" t="n">
+        <v>31.5967</v>
+      </c>
+      <c r="G368" t="n">
+        <v>48.0938</v>
+      </c>
+      <c r="H368" t="n">
+        <v>39.58</v>
+      </c>
+      <c r="I368" t="n">
+        <v>39.6648</v>
+      </c>
+      <c r="J368" t="n">
+        <v>39.1607</v>
+      </c>
+      <c r="K368" t="n">
+        <v>43.6975</v>
+      </c>
+      <c r="L368" t="n">
+        <v>39.27</v>
+      </c>
+      <c r="M368" t="n">
+        <v>40.8979</v>
+      </c>
+      <c r="N368" t="n">
+        <v>41.9604</v>
+      </c>
+      <c r="O368" t="n">
+        <v>28.1481</v>
+      </c>
       <c r="P368" t="n">
         <v>45.62</v>
       </c>
@@ -42625,18 +42969,42 @@
       <c r="C369" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="D369" t="inlineStr"/>
-      <c r="E369" t="inlineStr"/>
-      <c r="F369" t="inlineStr"/>
-      <c r="G369" t="inlineStr"/>
-      <c r="H369" t="inlineStr"/>
-      <c r="I369" t="inlineStr"/>
-      <c r="J369" t="inlineStr"/>
-      <c r="K369" t="inlineStr"/>
-      <c r="L369" t="inlineStr"/>
-      <c r="M369" t="inlineStr"/>
-      <c r="N369" t="inlineStr"/>
-      <c r="O369" t="inlineStr"/>
+      <c r="D369" t="n">
+        <v>40.18</v>
+      </c>
+      <c r="E369" t="n">
+        <v>35.0114</v>
+      </c>
+      <c r="F369" t="n">
+        <v>31.5619</v>
+      </c>
+      <c r="G369" t="n">
+        <v>48.8095</v>
+      </c>
+      <c r="H369" t="n">
+        <v>42.3</v>
+      </c>
+      <c r="I369" t="n">
+        <v>46.2271</v>
+      </c>
+      <c r="J369" t="n">
+        <v>47.6721</v>
+      </c>
+      <c r="K369" t="n">
+        <v>34.6667</v>
+      </c>
+      <c r="L369" t="n">
+        <v>47.73</v>
+      </c>
+      <c r="M369" t="n">
+        <v>50.051</v>
+      </c>
+      <c r="N369" t="n">
+        <v>50.6125</v>
+      </c>
+      <c r="O369" t="n">
+        <v>43.3121</v>
+      </c>
       <c r="P369" t="n">
         <v>56.5</v>
       </c>
@@ -45615,10 +45983,18 @@
       <c r="C395" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="D395" t="inlineStr"/>
-      <c r="E395" t="inlineStr"/>
-      <c r="F395" t="inlineStr"/>
-      <c r="G395" t="inlineStr"/>
+      <c r="D395" t="n">
+        <v>0.7552870090634441</v>
+      </c>
+      <c r="E395" t="n">
+        <v>0.1721170395869191</v>
+      </c>
+      <c r="F395" t="n">
+        <v>0</v>
+      </c>
+      <c r="G395" t="n">
+        <v>0.8605851979345955</v>
+      </c>
       <c r="H395" t="n">
         <v>0.5105740181268882</v>
       </c>
@@ -45722,10 +46098,18 @@
       <c r="C396" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D396" t="inlineStr"/>
-      <c r="E396" t="inlineStr"/>
-      <c r="F396" t="inlineStr"/>
-      <c r="G396" t="inlineStr"/>
+      <c r="D396" t="n">
+        <v>0.7522658610271903</v>
+      </c>
+      <c r="E396" t="n">
+        <v>0.1717241379310345</v>
+      </c>
+      <c r="F396" t="n">
+        <v>0</v>
+      </c>
+      <c r="G396" t="n">
+        <v>0.8586206896551725</v>
+      </c>
       <c r="H396" t="n">
         <v>0.5287009063444109</v>
       </c>
@@ -45829,10 +46213,18 @@
       <c r="C397" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D397" t="inlineStr"/>
-      <c r="E397" t="inlineStr"/>
-      <c r="F397" t="inlineStr"/>
-      <c r="G397" t="inlineStr"/>
+      <c r="D397" t="n">
+        <v>0.7583081570996979</v>
+      </c>
+      <c r="E397" t="n">
+        <v>0.1725085910652921</v>
+      </c>
+      <c r="F397" t="n">
+        <v>0</v>
+      </c>
+      <c r="G397" t="n">
+        <v>0.8625429553264605</v>
+      </c>
       <c r="H397" t="n">
         <v>0.5105740181268882</v>
       </c>
@@ -45845,10 +46237,18 @@
       <c r="K397" t="n">
         <v>0.6680327868852459</v>
       </c>
-      <c r="L397" t="inlineStr"/>
-      <c r="M397" t="inlineStr"/>
-      <c r="N397" t="inlineStr"/>
-      <c r="O397" t="inlineStr"/>
+      <c r="L397" t="n">
+        <v>0.2809667673716012</v>
+      </c>
+      <c r="M397" t="n">
+        <v>0.0760741594871029</v>
+      </c>
+      <c r="N397" t="n">
+        <v>0.0472194980204133</v>
+      </c>
+      <c r="O397" t="n">
+        <v>0.4223300970873786</v>
+      </c>
       <c r="P397" t="n">
         <v>0.7552870090634441</v>
       </c>
@@ -45873,10 +46273,18 @@
       <c r="W397" t="n">
         <v>0.7532467532467533</v>
       </c>
-      <c r="X397" t="inlineStr"/>
-      <c r="Y397" t="inlineStr"/>
-      <c r="Z397" t="inlineStr"/>
-      <c r="AA397" t="inlineStr"/>
+      <c r="X397" t="n">
+        <v>0.5770392749244713</v>
+      </c>
+      <c r="Y397" t="n">
+        <v>0.5994015463394461</v>
+      </c>
+      <c r="Z397" t="n">
+        <v>0.6069274327768243</v>
+      </c>
+      <c r="AA397" t="n">
+        <v>0.509090909090909</v>
+      </c>
       <c r="AB397" t="n">
         <v>0.7824773413897281</v>
       </c>
@@ -45920,10 +46328,18 @@
       <c r="C398" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="D398" t="inlineStr"/>
-      <c r="E398" t="inlineStr"/>
-      <c r="F398" t="inlineStr"/>
-      <c r="G398" t="inlineStr"/>
+      <c r="D398" t="n">
+        <v>0.7462235649546828</v>
+      </c>
+      <c r="E398" t="n">
+        <v>0.1709342560553633</v>
+      </c>
+      <c r="F398" t="n">
+        <v>0</v>
+      </c>
+      <c r="G398" t="n">
+        <v>0.8546712802768166</v>
+      </c>
       <c r="H398" t="n">
         <v>0.513595166163142</v>
       </c>
@@ -46027,10 +46443,18 @@
       <c r="C399" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="D399" t="inlineStr"/>
-      <c r="E399" t="inlineStr"/>
-      <c r="F399" t="inlineStr"/>
-      <c r="G399" t="inlineStr"/>
+      <c r="D399" t="n">
+        <v>0.743202416918429</v>
+      </c>
+      <c r="E399" t="n">
+        <v>0.1705372616984402</v>
+      </c>
+      <c r="F399" t="n">
+        <v>0</v>
+      </c>
+      <c r="G399" t="n">
+        <v>0.8526863084922011</v>
+      </c>
       <c r="H399" t="n">
         <v>0.4984894259818731</v>
       </c>

</xml_diff>